<commit_message>
Mejorar estilo de graficos: barras con degradado, cuadricula suave y etiquetas
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WJLznUNzeAdt4qXRWo1KFV
</commit_message>
<xml_diff>
--- a/ingreso-promedio/Ingreso_promedio_mensual_Nacional_Lima.xlsx
+++ b/ingreso-promedio/Ingreso_promedio_mensual_Nacional_Lima.xlsx
@@ -29,10 +29,12 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00404040"/>
       <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00404040"/>
     </font>
   </fonts>
   <fills count="3">
@@ -44,7 +46,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0FAFC"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,16 +60,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00D9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00D9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00D9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="00D9D9D9"/>
       </bottom>
     </border>
   </borders>
@@ -164,7 +166,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -172,11 +173,28 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1300" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="404040"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>Ingreso promedio mensual proveniente del trabajo - NACIONAL</a:t>
+              <a:rPr sz="1300" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="404040"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Ingreso promedio mensual proveniente del trabajo · NACIONAL</a:t>
             </a:r>
+            <a:endParaRPr sz="1300" b="1">
+              <a:solidFill>
+                <a:srgbClr val="404040"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:endParaRPr>
           </a:p>
         </rich>
       </tx>
@@ -189,10 +207,19 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="9E3A38"/>
-            </a:solidFill>
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:srgbClr val="D96B68"/>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:srgbClr val="8B2C2A"/>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="1"/>
+            </a:gradFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -209,9 +236,29 @@
         </ser>
         <dLbls>
           <numFmt formatCode="#,##0.0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="900" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="595959"/>
+                  </a:solidFill>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+            </a:p>
+          </txPr>
+          <dLblPos val="outEnd"/>
+          <showLegendKey val="0"/>
           <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
         </dLbls>
-        <gapWidth val="60"/>
+        <gapWidth val="55"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -220,24 +267,33 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Año</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
+              <a:srgbClr val="BFBFBF"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:solidFill>
+                  <a:srgbClr val="595959"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -245,38 +301,61 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <min val="0"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Soles</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="E6E6E6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:solidFill>
+                  <a:srgbClr val="595959"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -284,11 +363,28 @@
           <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1300" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="404040"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>Ingreso promedio mensual proveniente del trabajo - LIMA</a:t>
+              <a:rPr sz="1300" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="404040"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Ingreso promedio mensual proveniente del trabajo · LIMA</a:t>
             </a:r>
+            <a:endParaRPr sz="1300" b="1">
+              <a:solidFill>
+                <a:srgbClr val="404040"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:endParaRPr>
           </a:p>
         </rich>
       </tx>
@@ -301,10 +397,19 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="9E3A38"/>
-            </a:solidFill>
+            <a:gradFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:gsLst>
+                <a:gs pos="0">
+                  <a:srgbClr val="6FA8DC"/>
+                </a:gs>
+                <a:gs pos="100000">
+                  <a:srgbClr val="1F4E79"/>
+                </a:gs>
+              </a:gsLst>
+              <a:lin ang="5400000" scaled="1"/>
+            </a:gradFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -321,9 +426,29 @@
         </ser>
         <dLbls>
           <numFmt formatCode="#,##0.0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="900" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="595959"/>
+                  </a:solidFill>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t/>
+              </a:r>
+            </a:p>
+          </txPr>
+          <dLblPos val="outEnd"/>
+          <showLegendKey val="0"/>
           <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
         </dLbls>
-        <gapWidth val="60"/>
+        <gapWidth val="55"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -332,24 +457,33 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Año</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
+              <a:srgbClr val="BFBFBF"/>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:solidFill>
+                  <a:srgbClr val="595959"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -357,32 +491,56 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <min val="0"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Soles</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="E6E6E6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900">
+                <a:solidFill>
+                  <a:srgbClr val="595959"/>
+                </a:solidFill>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -395,7 +553,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="3960000"/>
+    <ext cx="8640000" cy="4140000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -414,10 +572,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>32</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="3960000"/>
+    <ext cx="8640000" cy="4140000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -727,7 +885,7 @@
   <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Actualizar graficos al rango 2010-2020
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WJLznUNzeAdt4qXRWo1KFV
</commit_message>
<xml_diff>
--- a/ingreso-promedio/Ingreso_promedio_mensual_Nacional_Lima.xlsx
+++ b/ingreso-promedio/Ingreso_promedio_mensual_Nacional_Lima.xlsx
@@ -902,37 +902,37 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>2008</v>
+        <v>2010</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>2009</v>
+        <v>2011</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2010</v>
+        <v>2012</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2011</v>
+        <v>2013</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2012</v>
+        <v>2014</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>2014</v>
+        <v>2016</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>2015</v>
+        <v>2017</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>2018</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="4">
@@ -942,37 +942,37 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>893.2</v>
+        <v>986.9</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>963.9</v>
+        <v>1069</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>986.9</v>
+        <v>1155.7</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>1069</v>
+        <v>1184.6</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>1155.7</v>
+        <v>1239.9</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>1184.6</v>
+        <v>1304.9</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1239.9</v>
+        <v>1370.7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1304.9</v>
+        <v>1376.8</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>1370.7</v>
+        <v>1400.1</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>1376.8</v>
+        <v>1443.1</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>1400.1</v>
+        <v>1268.8</v>
       </c>
     </row>
     <row r="5">
@@ -982,37 +982,37 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>1236.1</v>
+        <v>1285.8</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1296.8</v>
+        <v>1391.9</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>1285.8</v>
+        <v>1517.2</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>1391.9</v>
+        <v>1543.2</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1517.2</v>
+        <v>1640.4</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1543.2</v>
+        <v>1753.1</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>1640.4</v>
+        <v>1870</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>1753.1</v>
+        <v>1851.6</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>1870</v>
+        <v>1857.3</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>1851.6</v>
+        <v>1885.9</v>
       </c>
       <c r="L5" s="4" t="n">
-        <v>1857.3</v>
+        <v>1653.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>